<commit_message>
KPI actualizado 2026-07-08 20:55 UTC
</commit_message>
<xml_diff>
--- a/data/50001557 - ATACAMA KOZAN OT4340.xlsx
+++ b/data/50001557 - ATACAMA KOZAN OT4340.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1183" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="309">
   <si>
     <t xml:space="preserve"> 50001557 - ATACAMA KOZAN</t>
   </si>
@@ -4571,9 +4571,11 @@
       <c r="B53" s="8">
         <v>46169.558565775464</v>
       </c>
-      <c r="C53" s="9"/>
+      <c r="C53" s="8">
+        <v>46211.86420568287</v>
+      </c>
       <c r="D53" s="8">
-        <v>46169.61885943287</v>
+        <v>46211.86422231482</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>189</v>
@@ -4621,10 +4623,10 @@
         <v>32</v>
       </c>
       <c r="T53" s="9">
-        <v>0</v>
-      </c>
-      <c r="U53" s="11" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="U53" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4634,9 +4636,11 @@
       <c r="B54" s="5">
         <v>46169.55856972223</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46211.864191967594</v>
+      </c>
       <c r="D54" s="5">
-        <v>46206.486704027775</v>
+        <v>46211.86419394676</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>174</v>
@@ -5852,9 +5856,11 @@
       <c r="B74" s="5">
         <v>46169.55884254629</v>
       </c>
-      <c r="C74" s="6"/>
+      <c r="C74" s="5">
+        <v>46211.86404540509</v>
+      </c>
       <c r="D74" s="5">
-        <v>46206.48683333333</v>
+        <v>46211.86406403936</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>247</v>
@@ -5889,9 +5895,11 @@
       <c r="Q74" s="6"/>
       <c r="R74" s="6"/>
       <c r="S74" s="6"/>
-      <c r="T74" s="6"/>
-      <c r="U74" s="12" t="s">
-        <v>169</v>
+      <c r="T74" s="6">
+        <v>1</v>
+      </c>
+      <c r="U74" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -6570,7 +6578,7 @@
         <v>46206.486792916665</v>
       </c>
       <c r="D86" s="5">
-        <v>46206.48679516204</v>
+        <v>46211.86420142361</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>261</v>
@@ -6623,7 +6631,7 @@
       </c>
       <c r="C87" s="9"/>
       <c r="D87" s="8">
-        <v>46211.83096003473</v>
+        <v>46211.8640300463</v>
       </c>
       <c r="E87" s="9" t="s">
         <v>280</v>
@@ -6659,7 +6667,9 @@
       <c r="R87" s="9"/>
       <c r="S87" s="9"/>
       <c r="T87" s="9"/>
-      <c r="U87" s="9"/>
+      <c r="U87" s="12" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
@@ -7028,9 +7038,11 @@
       <c r="B94" s="5">
         <v>46169.55929686343</v>
       </c>
-      <c r="C94" s="6"/>
+      <c r="C94" s="5">
+        <v>46211.86400608796</v>
+      </c>
       <c r="D94" s="5">
-        <v>46196.573311342596</v>
+        <v>46211.86402001158</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>297</v>
@@ -7078,10 +7090,10 @@
         <v>32</v>
       </c>
       <c r="T94" s="6">
-        <v>0</v>
-      </c>
-      <c r="U94" s="11" t="s">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="U94" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -7091,9 +7103,11 @@
       <c r="B95" s="8">
         <v>46169.55930180555</v>
       </c>
-      <c r="C95" s="9"/>
+      <c r="C95" s="8">
+        <v>46211.863989895835</v>
+      </c>
       <c r="D95" s="8">
-        <v>46205.598038449076</v>
+        <v>46211.863992280094</v>
       </c>
       <c r="E95" s="9" t="s">
         <v>174</v>
@@ -7193,7 +7207,7 @@
       </c>
       <c r="C97" s="9"/>
       <c r="D97" s="8">
-        <v>46169.621991215274</v>
+        <v>46211.86403020834</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>304</v>
@@ -7243,8 +7257,8 @@
       <c r="T97" s="9">
         <v>0</v>
       </c>
-      <c r="U97" s="11" t="s">
-        <v>100</v>
+      <c r="U97" s="12" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
@@ -7256,7 +7270,7 @@
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46196.805673622686</v>
+        <v>46211.86403085648</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>308</v>
@@ -7306,8 +7320,8 @@
       <c r="T98" s="6">
         <v>0</v>
       </c>
-      <c r="U98" s="11" t="s">
-        <v>100</v>
+      <c r="U98" s="12" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-10 17:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001557 - ATACAMA KOZAN OT4340.xlsx
+++ b/data/50001557 - ATACAMA KOZAN OT4340.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="311">
   <si>
     <t xml:space="preserve"> 50001557 - ATACAMA KOZAN</t>
   </si>
@@ -119,6 +119,72 @@
   </si>
   <si>
     <t>Apertura pedido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buen día,
+Para el pedido 1557 se tienen 2 equipos ZVN 1-7-37/2, 2 equipos ZVN 1-7-30/2, 1 equipo ZVN 1-9-37/2 y 1 equipo JZR 6-18.5/2 para Atacama Kozan:
+    *    Planos para fabricación Ventilador ZVN 1-7-37/2 con motor OMEC
+        *    Incluye: Tobera + Rejilla
+        *    hgutierrez@zitron.com, tu apoyo con los planos.
+    *    Rodete:
+        *    Rodete monobloque GEL 7-37  
+        *    Código: 300065
+        *    Plano Mecanizado 3534.07.04.37.D55
+    *    Datos eléctricos para el motor:
+        *    Motor 37 KW, 2 Polos, Frame 200L.
+        *    380 VAC, 50 Hz, IEC, IP55, FS 1.0.-
+        *    Código: 350004
+--
+    *    Planos para fabricación Ventilador ZVN 1-7-30/2 con motor OMEC
+        *    Incluye: Tobera + Rejilla
+        *    hgutierrez@zitron.com, tu apoyo con los planos.
+    *    Rodete:
+        *    Rodete monobloque GEL 7-30
+        *    Código: 300062
+        *    Plano Mecanizado 3534.07.04.30.D55
+    *    Datos eléctricos para el motor:
+        *    Motor 30 KW, 2 Polos, Frame 200L.
+        *    380 VAC, 50 Hz, IEC, IP55, FS 1.0.-
+        *    Código: 350004
+        *    benjamin.bustos@zitron.com, se debe solicitar duplicado de placas.
+--
+    *    Planos para fabricación Ventilador ZVN 1-9-37/2 con motor OMEC
+        *    Incluye: Tobera + Rejilla
+        *    hgutierrez@zitron.com, tu apoyo con los planos.
+    *    Rodete:
+        *    Rodete de placas s/plano 4999.00
+        *    Alabe s/ plano 4999.01
+        *    Z8 N590
+        *    Código 300000
+        *    hgutierrez@zitron.com, tu apoyo con la definición de calaje
+    *    Datos eléctricos para el motor:
+        *    Motor 37 KW, 2 Polos, Frame 200L.
+        *    380 VAC, 50 Hz, IEC, IP55, FS 1.0.-
+        *    Código: 350004
+--
+    *    Fabricación Ventilador JZR 6-18.5/2 con motor WEG
+        *    Incluye: Tobera + Rejilla + 2FAR90/100 + Bastidor
+        *    Plano CH1463
+    *    Rodete:
+        *    Rodete monobloque GEL 6-15  
+        *    Código 300056
+        *    Plano Mecanizado 3534.06.04.15.D42
+    *    Datos eléctricos para el motor:
+        *    Motor 18.5 KW, 2 Polos, Frame 160L.
+        *    380 VAC, 50 Hz, IEC, IP55, FS 1.0.-
+--
+    *    Datos eléctricos para tableros:
+        *    Tablero YD  18.5kW, 380 VAC, 50 Hz, IP66.
+        *    Tablero YD  30kW, 380 VAC, 50 Hz, IP66.
+        *    Tablero YD  37kW, 380 VAC, 50 Hz, IP66.
+        *    Incluye luces piloto, botones y protección de entrada
+        *    Propuestas en sistema.
+    *    Tratamiento superficial estándar Zitron para todas las unidades:
+        *    Preparación de superficie: Arenado SSPC-SP10
+        *    1ª capa imprimación 60 micras Hempadur 15570 Color 12430
+        *    2ª capa intermedia 40 micras Hempathane HS 55610 Color 20450 RAL 9001
+    *    Fecha de entrega: 16-06-2026
+</t>
   </si>
   <si>
     <t>1215166329020201</t>
@@ -1723,7 +1789,7 @@
         <v>46181.62347399305</v>
       </c>
       <c r="D6" s="5">
-        <v>46181.624255925926</v>
+        <v>46213.7119689699</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1745,7 +1811,7 @@
         <v>26</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="M6" s="6" t="s">
         <v>26</v>
@@ -1777,7 +1843,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="8">
         <v>46169.55814432871</v>
@@ -1789,7 +1855,7 @@
         <v>46181.62349788194</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>26</v>
@@ -1808,7 +1874,7 @@
         <v>26</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M7" s="9" t="s">
         <v>26</v>
@@ -1840,7 +1906,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="5">
         <v>46169.55814774305</v>
@@ -1852,7 +1918,7 @@
         <v>46181.62350184028</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>26</v>
@@ -1871,7 +1937,7 @@
         <v>26</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M8" s="6" t="s">
         <v>26</v>
@@ -1883,7 +1949,7 @@
         <v>26</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q8" s="5">
         <v>46154</v>
@@ -1903,7 +1969,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9" s="8">
         <v>46169.55815164352</v>
@@ -1915,7 +1981,7 @@
         <v>46181.62350840278</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>26</v>
@@ -1934,7 +2000,7 @@
         <v>26</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="M9" s="9" t="s">
         <v>26</v>
@@ -1966,7 +2032,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B10" s="5">
         <v>46169.55800939815</v>
@@ -1978,7 +2044,7 @@
         <v>46197.83892112269</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>25</v>
@@ -2002,7 +2068,7 @@
         <v>26</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P10" s="6" t="s">
         <v>26</v>
@@ -2019,7 +2085,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="8">
         <v>46169.558185671296</v>
@@ -2031,16 +2097,16 @@
         <v>46196.80567361111</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I11" s="8">
         <v>46155</v>
@@ -2052,19 +2118,19 @@
         <v>26</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M11" s="9" t="s">
         <v>26</v>
       </c>
       <c r="N11" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O11" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q11" s="8">
         <v>46155</v>
@@ -2084,7 +2150,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="5">
         <v>46169.558191840275</v>
@@ -2096,16 +2162,16 @@
         <v>46196.80567332176</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I12" s="5">
         <v>46155</v>
@@ -2117,19 +2183,19 @@
         <v>26</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="Q12" s="5">
         <v>46155</v>
@@ -2149,7 +2215,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B13" s="8">
         <v>46169.558197418984</v>
@@ -2161,16 +2227,16 @@
         <v>46196.80567320602</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I13" s="8">
         <v>46155</v>
@@ -2188,13 +2254,13 @@
         <v>26</v>
       </c>
       <c r="N13" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P13" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="Q13" s="8">
         <v>46155</v>
@@ -2214,7 +2280,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B14" s="5">
         <v>46169.558013773145</v>
@@ -2226,7 +2292,7 @@
         <v>46190.64417138889</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>25</v>
@@ -2250,7 +2316,7 @@
         <v>26</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="P14" s="6" t="s">
         <v>26</v>
@@ -2267,7 +2333,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B15" s="8">
         <v>46169.558213564815</v>
@@ -2279,16 +2345,16 @@
         <v>46181.62446385417</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I15" s="8">
         <v>46157</v>
@@ -2306,13 +2372,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O15" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="Q15" s="8">
         <v>46157</v>
@@ -2332,7 +2398,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B16" s="5">
         <v>46169.558224479166</v>
@@ -2344,16 +2410,16 @@
         <v>46181.62447002315</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I16" s="5">
         <v>46167</v>
@@ -2371,13 +2437,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="Q16" s="5">
         <v>46167</v>
@@ -2397,7 +2463,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B17" s="8">
         <v>46169.558230821756</v>
@@ -2409,16 +2475,16 @@
         <v>46183.90651931713</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I17" s="8">
         <v>46167</v>
@@ -2436,13 +2502,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q17" s="8">
         <v>46167</v>
@@ -2462,7 +2528,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B18" s="5">
         <v>46169.55823646991</v>
@@ -2474,16 +2540,16 @@
         <v>46183.90665107639</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I18" s="5">
         <v>46239</v>
@@ -2501,13 +2567,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="Q18" s="5">
         <v>46239</v>
@@ -2527,7 +2593,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B19" s="8">
         <v>46169.55824171296</v>
@@ -2539,16 +2605,16 @@
         <v>46183.90666170139</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I19" s="8">
         <v>46239</v>
@@ -2566,13 +2632,13 @@
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="Q19" s="8">
         <v>46239</v>
@@ -2592,7 +2658,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B20" s="5">
         <v>46169.55824574074</v>
@@ -2604,16 +2670,16 @@
         <v>46190.64415820602</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I20" s="5">
         <v>46239</v>
@@ -2631,13 +2697,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Q20" s="5">
         <v>46239</v>
@@ -2657,7 +2723,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" s="8">
         <v>46169.55825006944</v>
@@ -2669,16 +2735,16 @@
         <v>46183.90735393518</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I21" s="8">
         <v>46239</v>
@@ -2696,13 +2762,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q21" s="8">
         <v>46239</v>
@@ -2722,7 +2788,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B22" s="5">
         <v>46169.55801826389</v>
@@ -2734,7 +2800,7 @@
         <v>46200.818425798614</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>25</v>
@@ -2758,7 +2824,7 @@
         <v>26</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P22" s="6" t="s">
         <v>26</v>
@@ -2771,7 +2837,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B23" s="8">
         <v>46169.558301956014</v>
@@ -2783,16 +2849,16 @@
         <v>46200.81833380787</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I23" s="8">
         <v>46169</v>
@@ -2810,13 +2876,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q23" s="8">
         <v>46169</v>
@@ -2836,7 +2902,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B24" s="5">
         <v>46169.558306516206</v>
@@ -2848,16 +2914,16 @@
         <v>46195.69079224537</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I24" s="5">
         <v>46169</v>
@@ -2875,13 +2941,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
@@ -2892,12 +2958,12 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B25" s="8">
         <v>46169.55831137732</v>
@@ -2909,16 +2975,16 @@
         <v>46195.690800474535</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I25" s="8">
         <v>46171</v>
@@ -2936,13 +3002,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q25" s="9"/>
       <c r="R25" s="9"/>
@@ -2953,12 +3019,12 @@
         <v>0</v>
       </c>
       <c r="U25" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B26" s="5">
         <v>46169.55831605324</v>
@@ -2970,16 +3036,16 @@
         <v>46212.20714363426</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I26" s="5">
         <v>46169</v>
@@ -2997,13 +3063,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q26" s="5">
         <v>46169</v>
@@ -3012,7 +3078,7 @@
         <v>46219</v>
       </c>
       <c r="S26" s="12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="T26" s="6">
         <v>1</v>
@@ -3023,7 +3089,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B27" s="8">
         <v>46169.55832063657</v>
@@ -3035,16 +3101,16 @@
         <v>46184.7364097338</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I27" s="8">
         <v>46169</v>
@@ -3062,13 +3128,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
@@ -3079,12 +3145,12 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B28" s="5">
         <v>46169.55832539352</v>
@@ -3096,16 +3162,16 @@
         <v>46184.736449375</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I28" s="5">
         <v>46171</v>
@@ -3123,13 +3189,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3140,12 +3206,12 @@
         <v>0</v>
       </c>
       <c r="U28" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B29" s="8">
         <v>46169.55833006944</v>
@@ -3157,16 +3223,16 @@
         <v>46200.81836952546</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I29" s="8">
         <v>46161</v>
@@ -3184,13 +3250,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q29" s="8">
         <v>46161</v>
@@ -3210,7 +3276,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B30" s="5">
         <v>46169.55833486111</v>
@@ -3222,16 +3288,16 @@
         <v>46195.69066259259</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I30" s="5">
         <v>46161</v>
@@ -3249,13 +3315,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3266,12 +3332,12 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B31" s="8">
         <v>46169.5583402662</v>
@@ -3283,16 +3349,16 @@
         <v>46195.69066760417</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I31" s="8">
         <v>46178</v>
@@ -3310,13 +3376,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
@@ -3327,12 +3393,12 @@
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B32" s="5">
         <v>46169.55834503472</v>
@@ -3344,16 +3410,16 @@
         <v>46195.6906680324</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I32" s="5">
         <v>46178</v>
@@ -3371,13 +3437,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3388,12 +3454,12 @@
         <v>0</v>
       </c>
       <c r="U32" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B33" s="8">
         <v>46169.55836335648</v>
@@ -3405,16 +3471,16 @@
         <v>46184.532641875005</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I33" s="8">
         <v>46241</v>
@@ -3432,13 +3498,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="Q33" s="8">
         <v>46241</v>
@@ -3458,7 +3524,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B34" s="5">
         <v>46169.558367986116</v>
@@ -3470,16 +3536,16 @@
         <v>46184.53245875</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I34" s="5">
         <v>46241</v>
@@ -3497,13 +3563,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
@@ -3514,12 +3580,12 @@
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B35" s="8">
         <v>46169.55837292824</v>
@@ -3531,16 +3597,16 @@
         <v>46184.532615856486</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I35" s="8">
         <v>46245</v>
@@ -3558,13 +3624,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
@@ -3575,12 +3641,12 @@
         <v>0</v>
       </c>
       <c r="U35" s="11" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B36" s="5">
         <v>46169.55837825232</v>
@@ -3592,16 +3658,16 @@
         <v>46184.53258194444</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I36" s="5">
         <v>46241</v>
@@ -3619,10 +3685,10 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>26</v>
@@ -3645,7 +3711,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B37" s="8">
         <v>46169.558381979165</v>
@@ -3657,16 +3723,16 @@
         <v>46184.5322071875</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I37" s="8">
         <v>46241</v>
@@ -3684,13 +3750,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
@@ -3700,7 +3766,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B38" s="5">
         <v>46169.55838657408</v>
@@ -3712,16 +3778,16 @@
         <v>46184.53255631945</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I38" s="5">
         <v>46245</v>
@@ -3739,13 +3805,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3755,7 +3821,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B39" s="8">
         <v>46169.55839107639</v>
@@ -3767,16 +3833,16 @@
         <v>46205.600326053245</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I39" s="8">
         <v>46241</v>
@@ -3794,10 +3860,10 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>26</v>
@@ -3820,7 +3886,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B40" s="5">
         <v>46169.55839478009</v>
@@ -3832,16 +3898,16 @@
         <v>46195.70360162037</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I40" s="5">
         <v>46241</v>
@@ -3859,13 +3925,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -3875,7 +3941,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B41" s="8">
         <v>46169.55839910879</v>
@@ -3887,16 +3953,16 @@
         <v>46195.70375376157</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I41" s="8">
         <v>46252</v>
@@ -3914,13 +3980,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="Q41" s="9"/>
       <c r="R41" s="9"/>
@@ -3930,7 +3996,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B42" s="5">
         <v>46169.55840355324</v>
@@ -3942,16 +4008,16 @@
         <v>46205.59994755787</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I42" s="5">
         <v>46281</v>
@@ -3969,10 +4035,10 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>26</v>
@@ -3985,7 +4051,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B43" s="8">
         <v>46169.55840677083</v>
@@ -3997,16 +4063,16 @@
         <v>46191.53701371528</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I43" s="8">
         <v>46241</v>
@@ -4024,10 +4090,10 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="P43" s="9" t="s">
         <v>26</v>
@@ -4050,7 +4116,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B44" s="5">
         <v>46169.55841037037</v>
@@ -4062,16 +4128,16 @@
         <v>46191.53679194444</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I44" s="5">
         <v>46241</v>
@@ -4089,13 +4155,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4105,7 +4171,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B45" s="8">
         <v>46169.558458217594</v>
@@ -4117,16 +4183,16 @@
         <v>46191.53698841435</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H45" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I45" s="8">
         <v>46245</v>
@@ -4144,13 +4210,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
@@ -4160,7 +4226,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B46" s="5">
         <v>46169.5584643287</v>
@@ -4170,7 +4236,7 @@
         <v>46182.75962331019</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>25</v>
@@ -4194,7 +4260,7 @@
         <v>26</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>26</v>
@@ -4204,12 +4270,12 @@
       <c r="S46" s="6"/>
       <c r="T46" s="6"/>
       <c r="U46" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B47" s="8">
         <v>46169.55846813657</v>
@@ -4221,16 +4287,16 @@
         <v>46197.715420312496</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I47" s="8">
         <v>46167</v>
@@ -4248,13 +4314,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Q47" s="8">
         <v>46167</v>
@@ -4263,7 +4329,7 @@
         <v>46184</v>
       </c>
       <c r="S47" s="11" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T47" s="9">
         <v>1</v>
@@ -4274,7 +4340,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B48" s="5">
         <v>46169.558472766206</v>
@@ -4286,16 +4352,16 @@
         <v>46181.72663056713</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I48" s="5">
         <v>46167</v>
@@ -4313,13 +4379,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Q48" s="6"/>
       <c r="R48" s="6"/>
@@ -4329,7 +4395,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B49" s="8">
         <v>46169.55849938658</v>
@@ -4341,16 +4407,16 @@
         <v>46197.71545016204</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I49" s="8">
         <v>46218</v>
@@ -4368,13 +4434,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P49" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="Q49" s="8">
         <v>46218</v>
@@ -4394,7 +4460,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B50" s="5">
         <v>46169.55850371528</v>
@@ -4406,16 +4472,16 @@
         <v>46195.690583055555</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I50" s="5">
         <v>46218</v>
@@ -4433,13 +4499,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
@@ -4449,7 +4515,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B51" s="8">
         <v>46169.55853228009</v>
@@ -4461,16 +4527,16 @@
         <v>46182.759871076385</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I51" s="8">
         <v>46238</v>
@@ -4488,13 +4554,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P51" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="Q51" s="8">
         <v>46238</v>
@@ -4514,7 +4580,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B52" s="5">
         <v>46169.55854641204</v>
@@ -4526,16 +4592,16 @@
         <v>46182.75984881945</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I52" s="5">
         <v>46238</v>
@@ -4553,13 +4619,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
@@ -4569,7 +4635,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B53" s="8">
         <v>46169.558565775464</v>
@@ -4581,16 +4647,16 @@
         <v>46211.86422231482</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I53" s="8">
         <v>46331</v>
@@ -4608,10 +4674,10 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P53" s="9" t="s">
         <v>26</v>
@@ -4634,7 +4700,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B54" s="5">
         <v>46169.55856972223</v>
@@ -4646,16 +4712,16 @@
         <v>46211.86419394676</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I54" s="5">
         <v>46331</v>
@@ -4673,13 +4739,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
@@ -4689,7 +4755,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B55" s="8">
         <v>46169.558586307874</v>
@@ -4701,7 +4767,7 @@
         <v>46198.597746307874</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>25</v>
@@ -4725,7 +4791,7 @@
         <v>26</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="P55" s="9" t="s">
         <v>26</v>
@@ -4742,7 +4808,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B56" s="5">
         <v>46169.55858945602</v>
@@ -4754,16 +4820,16 @@
         <v>46197.83559606482</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I56" s="5">
         <v>46254</v>
@@ -4781,13 +4847,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Q56" s="5">
         <v>46254</v>
@@ -4807,7 +4873,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B57" s="8">
         <v>46169.55859488426</v>
@@ -4819,16 +4885,16 @@
         <v>46197.85937331019</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I57" s="8">
         <v>46258</v>
@@ -4846,13 +4912,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P57" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Q57" s="8">
         <v>46258</v>
@@ -4872,7 +4938,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B58" s="5">
         <v>46169.55860118056</v>
@@ -4884,16 +4950,16 @@
         <v>46198.59771457176</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I58" s="5">
         <v>46254</v>
@@ -4911,13 +4977,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q58" s="5">
         <v>46254</v>
@@ -4937,7 +5003,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B59" s="8">
         <v>46169.55860636574</v>
@@ -4949,16 +5015,16 @@
         <v>46198.597709444446</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I59" s="8">
         <v>46258</v>
@@ -4976,13 +5042,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P59" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q59" s="8">
         <v>46258</v>
@@ -4997,12 +5063,12 @@
         <v>1</v>
       </c>
       <c r="U59" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B60" s="5">
         <v>46169.558650127314</v>
@@ -5014,16 +5080,16 @@
         <v>46198.59773310185</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I60" s="5">
         <v>46254</v>
@@ -5041,13 +5107,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Q60" s="5">
         <v>46254</v>
@@ -5067,7 +5133,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B61" s="8">
         <v>46169.55865608796</v>
@@ -5079,16 +5145,16 @@
         <v>46198.59773317129</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I61" s="8">
         <v>46258</v>
@@ -5106,13 +5172,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="P61" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q61" s="8">
         <v>46258</v>
@@ -5127,12 +5193,12 @@
         <v>1</v>
       </c>
       <c r="U61" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B62" s="5">
         <v>46169.55866105324</v>
@@ -5144,7 +5210,7 @@
         <v>46198.68229049769</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>25</v>
@@ -5168,7 +5234,7 @@
         <v>26</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>26</v>
@@ -5185,7 +5251,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B63" s="8">
         <v>46169.55866469907</v>
@@ -5197,16 +5263,16 @@
         <v>46197.85915361111</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I63" s="8">
         <v>46260</v>
@@ -5224,13 +5290,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q63" s="8">
         <v>46260</v>
@@ -5250,7 +5316,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B64" s="5">
         <v>46169.55867099537</v>
@@ -5262,16 +5328,16 @@
         <v>46197.85936673611</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I64" s="5">
         <v>46260</v>
@@ -5289,13 +5355,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
@@ -5305,7 +5371,7 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B65" s="8">
         <v>46169.558703518516</v>
@@ -5317,16 +5383,16 @@
         <v>46197.85387390046</v>
       </c>
       <c r="E65" s="9" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F65" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I65" s="8">
         <v>46269</v>
@@ -5344,13 +5410,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="O65" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P65" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q65" s="8">
         <v>46269</v>
@@ -5365,12 +5431,12 @@
         <v>1</v>
       </c>
       <c r="U65" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B66" s="5">
         <v>46169.55870879629</v>
@@ -5382,16 +5448,16 @@
         <v>46197.85915420139</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I66" s="5">
         <v>46269</v>
@@ -5409,13 +5475,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Q66" s="6"/>
       <c r="R66" s="6"/>
@@ -5425,7 +5491,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B67" s="8">
         <v>46169.558740625</v>
@@ -5437,16 +5503,16 @@
         <v>46205.65959174768</v>
       </c>
       <c r="E67" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F67" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I67" s="8">
         <v>46274</v>
@@ -5464,13 +5530,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="O67" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P67" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q67" s="8">
         <v>46274</v>
@@ -5485,12 +5551,12 @@
         <v>1</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B68" s="5">
         <v>46169.558745243055</v>
@@ -5502,16 +5568,16 @@
         <v>46205.659588587965</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I68" s="5">
         <v>46274</v>
@@ -5529,13 +5595,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="O68" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="P68" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Q68" s="6"/>
       <c r="R68" s="6"/>
@@ -5545,7 +5611,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B69" s="8">
         <v>46169.55876947917</v>
@@ -5557,7 +5623,7 @@
         <v>46211.70953918982</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>25</v>
@@ -5581,7 +5647,7 @@
         <v>26</v>
       </c>
       <c r="O69" s="9" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="P69" s="9" t="s">
         <v>26</v>
@@ -5594,7 +5660,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B70" s="5">
         <v>46169.55880633101</v>
@@ -5606,16 +5672,16 @@
         <v>46200.8197621875</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I70" s="5">
         <v>46220</v>
@@ -5633,13 +5699,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P70" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="Q70" s="5">
         <v>46220</v>
@@ -5659,7 +5725,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B71" s="8">
         <v>46169.5588177662</v>
@@ -5671,16 +5737,16 @@
         <v>46200.819831597226</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I71" s="8">
         <v>46325</v>
@@ -5698,13 +5764,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O71" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="P71" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="Q71" s="8">
         <v>46325</v>
@@ -5713,7 +5779,7 @@
         <v>46325</v>
       </c>
       <c r="S71" s="11" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="T71" s="9">
         <v>1</v>
@@ -5724,7 +5790,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B72" s="5">
         <v>46169.55882295139</v>
@@ -5736,16 +5802,16 @@
         <v>46200.81928909722</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I72" s="5">
         <v>46293</v>
@@ -5763,13 +5829,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Q72" s="5">
         <v>46293</v>
@@ -5789,7 +5855,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B73" s="8">
         <v>46169.55882788195</v>
@@ -5801,16 +5867,16 @@
         <v>46211.7093043287</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I73" s="8">
         <v>46282</v>
@@ -5828,13 +5894,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P73" s="9" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="Q73" s="8">
         <v>46282</v>
@@ -5854,7 +5920,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B74" s="5">
         <v>46169.55884254629</v>
@@ -5866,7 +5932,7 @@
         <v>46211.86406403936</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>25</v>
@@ -5890,7 +5956,7 @@
         <v>26</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="P74" s="6" t="s">
         <v>26</v>
@@ -5907,7 +5973,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B75" s="8">
         <v>46169.55884548611</v>
@@ -5919,16 +5985,16 @@
         <v>46211.70929236111</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I75" s="8">
         <v>46276</v>
@@ -5946,13 +6012,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="O75" s="9" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q75" s="8">
         <v>46276</v>
@@ -5967,12 +6033,12 @@
         <v>1</v>
       </c>
       <c r="U75" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B76" s="5">
         <v>46169.55884993056</v>
@@ -5984,16 +6050,16 @@
         <v>46211.70929407407</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I76" s="5">
         <v>46276</v>
@@ -6011,13 +6077,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Q76" s="6"/>
       <c r="R76" s="6"/>
@@ -6027,7 +6093,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B77" s="8">
         <v>46169.55893170139</v>
@@ -6039,16 +6105,16 @@
         <v>46197.495185555556</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H77" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I77" s="8">
         <v>46296</v>
@@ -6066,13 +6132,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q77" s="8">
         <v>46296</v>
@@ -6092,7 +6158,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B78" s="5">
         <v>46169.55893543981</v>
@@ -6104,16 +6170,16 @@
         <v>46204.879924837966</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I78" s="5">
         <v>46296</v>
@@ -6131,13 +6197,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="Q78" s="6"/>
       <c r="R78" s="6"/>
@@ -6147,7 +6213,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B79" s="8">
         <v>46169.558869560184</v>
@@ -6159,16 +6225,16 @@
         <v>46204.87981377315</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G79" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H79" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I79" s="8">
         <v>46328</v>
@@ -6186,13 +6252,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q79" s="8">
         <v>46328</v>
@@ -6212,7 +6278,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B80" s="5">
         <v>46169.55887296297</v>
@@ -6224,16 +6290,16 @@
         <v>46204.87978310185</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I80" s="5">
         <v>46328</v>
@@ -6251,13 +6317,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q80" s="6"/>
       <c r="R80" s="6"/>
@@ -6267,7 +6333,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B81" s="8">
         <v>46169.5589025463</v>
@@ -6279,16 +6345,16 @@
         <v>46204.880057013885</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H81" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I81" s="8">
         <v>46329</v>
@@ -6306,13 +6372,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q81" s="8">
         <v>46329</v>
@@ -6332,7 +6398,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B82" s="5">
         <v>46169.55890609954</v>
@@ -6344,16 +6410,16 @@
         <v>46204.87991711806</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I82" s="5">
         <v>46329</v>
@@ -6371,13 +6437,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q82" s="6"/>
       <c r="R82" s="6"/>
@@ -6387,7 +6453,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B83" s="8">
         <v>46169.55900443287</v>
@@ -6399,16 +6465,16 @@
         <v>46206.48671975694</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I83" s="8">
         <v>46330</v>
@@ -6426,13 +6492,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="O83" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P83" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q83" s="8">
         <v>46330</v>
@@ -6452,7 +6518,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B84" s="5">
         <v>46169.55901002315</v>
@@ -6464,16 +6530,16 @@
         <v>46206.48669563657</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I84" s="5">
         <v>46330</v>
@@ -6491,13 +6557,13 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P84" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q84" s="6"/>
       <c r="R84" s="6"/>
@@ -6507,7 +6573,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B85" s="8">
         <v>46169.55904462963</v>
@@ -6519,16 +6585,16 @@
         <v>46206.48682021991</v>
       </c>
       <c r="E85" s="9" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F85" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H85" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I85" s="8">
         <v>46332</v>
@@ -6546,13 +6612,13 @@
         <v>26</v>
       </c>
       <c r="N85" s="9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="O85" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="P85" s="9" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="Q85" s="8">
         <v>46332</v>
@@ -6572,7 +6638,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B86" s="5">
         <v>46169.559050138894</v>
@@ -6584,16 +6650,16 @@
         <v>46211.86420142361</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I86" s="5">
         <v>46332</v>
@@ -6611,13 +6677,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Q86" s="6"/>
       <c r="R86" s="6"/>
@@ -6627,7 +6693,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B87" s="8">
         <v>46169.55907484954</v>
@@ -6637,7 +6703,7 @@
         <v>46211.8640300463</v>
       </c>
       <c r="E87" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F87" s="9" t="s">
         <v>25</v>
@@ -6661,7 +6727,7 @@
         <v>26</v>
       </c>
       <c r="O87" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="P87" s="9" t="s">
         <v>26</v>
@@ -6671,12 +6737,12 @@
       <c r="S87" s="9"/>
       <c r="T87" s="9"/>
       <c r="U87" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B88" s="5">
         <v>46169.55907863426</v>
@@ -6688,16 +6754,16 @@
         <v>46211.70008446759</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I88" s="5">
         <v>46335</v>
@@ -6715,13 +6781,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q88" s="5">
         <v>46335</v>
@@ -6741,7 +6807,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="7" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B89" s="8">
         <v>46169.55908684028</v>
@@ -6753,16 +6819,16 @@
         <v>46211.700054201385</v>
       </c>
       <c r="E89" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F89" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="H89" s="9" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I89" s="8">
         <v>46335</v>
@@ -6780,13 +6846,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="O89" s="9" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="P89" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q89" s="9"/>
       <c r="R89" s="9"/>
@@ -6796,7 +6862,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B90" s="5">
         <v>46169.55918673611</v>
@@ -6808,16 +6874,16 @@
         <v>46211.83096391204</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I90" s="5">
         <v>46336</v>
@@ -6835,13 +6901,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O90" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P90" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q90" s="5">
         <v>46336</v>
@@ -6861,7 +6927,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B91" s="8">
         <v>46169.55919113426</v>
@@ -6873,16 +6939,16 @@
         <v>46211.83093474537</v>
       </c>
       <c r="E91" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F91" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H91" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I91" s="8">
         <v>46336</v>
@@ -6900,13 +6966,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="O91" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P91" s="9" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q91" s="9"/>
       <c r="R91" s="9"/>
@@ -6916,7 +6982,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B92" s="5">
         <v>46169.559239560185</v>
@@ -6928,16 +6994,16 @@
         <v>46197.859819363424</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I92" s="5">
         <v>46337</v>
@@ -6955,13 +7021,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q92" s="5">
         <v>46337</v>
@@ -6976,12 +7042,12 @@
         <v>1</v>
       </c>
       <c r="U92" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="7" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B93" s="8">
         <v>46169.559243842596</v>
@@ -6993,16 +7059,16 @@
         <v>46211.830942650464</v>
       </c>
       <c r="E93" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F93" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G93" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H93" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I93" s="8">
         <v>46337</v>
@@ -7020,13 +7086,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="O93" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P93" s="9" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="Q93" s="9"/>
       <c r="R93" s="9"/>
@@ -7036,7 +7102,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B94" s="5">
         <v>46169.55929686343</v>
@@ -7048,16 +7114,16 @@
         <v>46211.86402001158</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I94" s="5">
         <v>46338</v>
@@ -7075,13 +7141,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="O94" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P94" s="6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="Q94" s="5">
         <v>46338</v>
@@ -7101,7 +7167,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="7" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B95" s="8">
         <v>46169.55930180555</v>
@@ -7113,16 +7179,16 @@
         <v>46211.863992280094</v>
       </c>
       <c r="E95" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F95" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H95" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I95" s="8">
         <v>46338</v>
@@ -7140,13 +7206,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="O95" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="P95" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="Q95" s="9"/>
       <c r="R95" s="9"/>
@@ -7156,7 +7222,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B96" s="5">
         <v>46169.55938721065</v>
@@ -7166,7 +7232,7 @@
         <v>46169.60672822916</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>25</v>
@@ -7190,7 +7256,7 @@
         <v>26</v>
       </c>
       <c r="O96" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="P96" s="6" t="s">
         <v>26</v>
@@ -7203,7 +7269,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B97" s="8">
         <v>46169.55939094907</v>
@@ -7213,16 +7279,16 @@
         <v>46211.86403020834</v>
       </c>
       <c r="E97" s="9" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F97" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G97" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H97" s="9" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="I97" s="8">
         <v>46339</v>
@@ -7240,13 +7306,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="9" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="O97" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="P97" s="9" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Q97" s="8">
         <v>46339</v>
@@ -7261,12 +7327,12 @@
         <v>0</v>
       </c>
       <c r="U97" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B98" s="5">
         <v>46169.55939643519</v>
@@ -7276,16 +7342,16 @@
         <v>46211.86403085648</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I98" s="5">
         <v>46339</v>
@@ -7303,13 +7369,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Q98" s="5">
         <v>46339</v>
@@ -7324,7 +7390,7 @@
         <v>0</v>
       </c>
       <c r="U98" s="12" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>